<commit_message>
Remove report annotations and origin columns
</commit_message>
<xml_diff>
--- a/forms/survey-after.xlsx
+++ b/forms/survey-after.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey_responses" sheetId="1" r:id="R3a4c0ab0f2474dd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="2" r:id="Re347f95f5fd7406c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey_responses" sheetId="1" r:id="R6cd1f70ba0e649dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="2" r:id="Rfeac44bfcb154549"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -410,7 +410,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R905b937269ea41a9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R97fa6881e84c442d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -437,9 +437,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="surveyresponsesExport" displayName="surveyresponsesExport" ref="A1:I101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:I101"/>
-  <x:tableColumns count="9">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="surveyresponsesExport" displayName="surveyresponsesExport" ref="A1:H101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:H101"/>
+  <x:tableColumns count="8">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="response_date"/>
     <x:tableColumn id="3" name="age"/>
@@ -448,7 +448,6 @@
     <x:tableColumn id="6" name="named_peoples_count"/>
     <x:tableColumn id="7" name="is_aware"/>
     <x:tableColumn id="8" name="interested_in_events"/>
-    <x:tableColumn id="9" name="data_origin"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -660,7 +659,6 @@
     <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -685,11 +683,8 @@
       <x:c r="G1" s="11" t="str">
         <x:v>is_aware</x:v>
       </x:c>
-      <x:c r="H1" s="11" t="str">
+      <x:c r="H1" s="12" t="str">
         <x:v>interested_in_events</x:v>
-      </x:c>
-      <x:c r="I1" s="12" t="str">
-        <x:v>data_origin</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="23" customHeight="1">
@@ -717,9 +712,6 @@
       <x:c r="H2" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I2" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="3" t="str">
@@ -746,9 +738,6 @@
       <x:c r="H3" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I3" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="4" ht="23" customHeight="1">
       <x:c r="A4" s="3" t="str">
@@ -775,9 +764,6 @@
       <x:c r="H4" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I4" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="5" ht="23" customHeight="1">
       <x:c r="A5" s="3" t="str">
@@ -804,9 +790,6 @@
       <x:c r="H5" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I5" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
       <x:c r="A6" s="3" t="str">
@@ -833,9 +816,6 @@
       <x:c r="H6" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I6" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
       <x:c r="A7" s="3" t="str">
@@ -862,9 +842,6 @@
       <x:c r="H7" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I7" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="8" ht="23" customHeight="1">
       <x:c r="A8" s="3" t="str">
@@ -891,9 +868,6 @@
       <x:c r="H8" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I8" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="9" ht="23" customHeight="1">
       <x:c r="A9" s="3" t="str">
@@ -920,9 +894,6 @@
       <x:c r="H9" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I9" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
       <x:c r="A10" s="3" t="str">
@@ -949,9 +920,6 @@
       <x:c r="H10" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I10" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="11" ht="23" customHeight="1">
       <x:c r="A11" s="3" t="str">
@@ -978,9 +946,6 @@
       <x:c r="H11" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I11" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
       <x:c r="A12" s="3" t="str">
@@ -1007,9 +972,6 @@
       <x:c r="H12" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I12" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
       <x:c r="A13" s="3" t="str">
@@ -1036,9 +998,6 @@
       <x:c r="H13" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I13" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
       <x:c r="A14" s="3" t="str">
@@ -1065,9 +1024,6 @@
       <x:c r="H14" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I14" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
       <x:c r="A15" s="3" t="str">
@@ -1094,9 +1050,6 @@
       <x:c r="H15" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I15" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
       <x:c r="A16" s="3" t="str">
@@ -1123,9 +1076,6 @@
       <x:c r="H16" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I16" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
       <x:c r="A17" s="3" t="str">
@@ -1152,9 +1102,6 @@
       <x:c r="H17" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I17" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
       <x:c r="A18" s="3" t="str">
@@ -1181,9 +1128,6 @@
       <x:c r="H18" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I18" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
       <x:c r="A19" s="3" t="str">
@@ -1210,9 +1154,6 @@
       <x:c r="H19" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I19" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
       <x:c r="A20" s="3" t="str">
@@ -1239,9 +1180,6 @@
       <x:c r="H20" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I20" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
       <x:c r="A21" s="3" t="str">
@@ -1268,9 +1206,6 @@
       <x:c r="H21" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I21" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
       <x:c r="A22" s="3" t="str">
@@ -1297,9 +1232,6 @@
       <x:c r="H22" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I22" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
       <x:c r="A23" s="3" t="str">
@@ -1326,9 +1258,6 @@
       <x:c r="H23" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I23" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
       <x:c r="A24" s="3" t="str">
@@ -1355,9 +1284,6 @@
       <x:c r="H24" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I24" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
       <x:c r="A25" s="3" t="str">
@@ -1384,9 +1310,6 @@
       <x:c r="H25" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I25" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
       <x:c r="A26" s="3" t="str">
@@ -1413,9 +1336,6 @@
       <x:c r="H26" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I26" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
       <x:c r="A27" s="3" t="str">
@@ -1442,9 +1362,6 @@
       <x:c r="H27" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I27" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
       <x:c r="A28" s="3" t="str">
@@ -1471,9 +1388,6 @@
       <x:c r="H28" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I28" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
       <x:c r="A29" s="3" t="str">
@@ -1500,9 +1414,6 @@
       <x:c r="H29" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I29" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="30" ht="23" customHeight="1">
       <x:c r="A30" s="3" t="str">
@@ -1529,9 +1440,6 @@
       <x:c r="H30" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I30" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="31" ht="23" customHeight="1">
       <x:c r="A31" s="3" t="str">
@@ -1558,9 +1466,6 @@
       <x:c r="H31" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I31" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="32" ht="23" customHeight="1">
       <x:c r="A32" s="3" t="str">
@@ -1587,9 +1492,6 @@
       <x:c r="H32" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I32" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="33" ht="23" customHeight="1">
       <x:c r="A33" s="3" t="str">
@@ -1616,9 +1518,6 @@
       <x:c r="H33" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I33" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="3" t="str">
@@ -1645,9 +1544,6 @@
       <x:c r="H34" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I34" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="35" ht="23" customHeight="1">
       <x:c r="A35" s="3" t="str">
@@ -1674,9 +1570,6 @@
       <x:c r="H35" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I35" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="36" ht="23" customHeight="1">
       <x:c r="A36" s="3" t="str">
@@ -1703,9 +1596,6 @@
       <x:c r="H36" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I36" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="37" ht="23" customHeight="1">
       <x:c r="A37" s="3" t="str">
@@ -1732,9 +1622,6 @@
       <x:c r="H37" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I37" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="38" ht="23" customHeight="1">
       <x:c r="A38" s="3" t="str">
@@ -1761,9 +1648,6 @@
       <x:c r="H38" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I38" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="39" ht="23" customHeight="1">
       <x:c r="A39" s="3" t="str">
@@ -1790,9 +1674,6 @@
       <x:c r="H39" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I39" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="40" ht="23" customHeight="1">
       <x:c r="A40" s="3" t="str">
@@ -1819,9 +1700,6 @@
       <x:c r="H40" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I40" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="41" ht="23" customHeight="1">
       <x:c r="A41" s="3" t="str">
@@ -1848,9 +1726,6 @@
       <x:c r="H41" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I41" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="42" ht="23" customHeight="1">
       <x:c r="A42" s="3" t="str">
@@ -1877,9 +1752,6 @@
       <x:c r="H42" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I42" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="43" ht="23" customHeight="1">
       <x:c r="A43" s="3" t="str">
@@ -1906,9 +1778,6 @@
       <x:c r="H43" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I43" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="44" ht="23" customHeight="1">
       <x:c r="A44" s="3" t="str">
@@ -1935,9 +1804,6 @@
       <x:c r="H44" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I44" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="45" ht="23" customHeight="1">
       <x:c r="A45" s="3" t="str">
@@ -1964,9 +1830,6 @@
       <x:c r="H45" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I45" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="46" ht="23" customHeight="1">
       <x:c r="A46" s="3" t="str">
@@ -1993,9 +1856,6 @@
       <x:c r="H46" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I46" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="47" ht="23" customHeight="1">
       <x:c r="A47" s="3" t="str">
@@ -2022,9 +1882,6 @@
       <x:c r="H47" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I47" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="48" ht="23" customHeight="1">
       <x:c r="A48" s="3" t="str">
@@ -2051,9 +1908,6 @@
       <x:c r="H48" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I48" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="49" ht="23" customHeight="1">
       <x:c r="A49" s="3" t="str">
@@ -2080,9 +1934,6 @@
       <x:c r="H49" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I49" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="50" ht="23" customHeight="1">
       <x:c r="A50" s="3" t="str">
@@ -2109,9 +1960,6 @@
       <x:c r="H50" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I50" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="51" ht="23" customHeight="1">
       <x:c r="A51" s="3" t="str">
@@ -2138,9 +1986,6 @@
       <x:c r="H51" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I51" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="52" ht="23" customHeight="1">
       <x:c r="A52" s="3" t="str">
@@ -2167,9 +2012,6 @@
       <x:c r="H52" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I52" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="53" ht="23" customHeight="1">
       <x:c r="A53" s="3" t="str">
@@ -2196,9 +2038,6 @@
       <x:c r="H53" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I53" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="54" ht="23" customHeight="1">
       <x:c r="A54" s="3" t="str">
@@ -2225,9 +2064,6 @@
       <x:c r="H54" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I54" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="55" ht="23" customHeight="1">
       <x:c r="A55" s="3" t="str">
@@ -2254,9 +2090,6 @@
       <x:c r="H55" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I55" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="56" ht="23" customHeight="1">
       <x:c r="A56" s="3" t="str">
@@ -2283,9 +2116,6 @@
       <x:c r="H56" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I56" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="57" ht="23" customHeight="1">
       <x:c r="A57" s="3" t="str">
@@ -2312,9 +2142,6 @@
       <x:c r="H57" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I57" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="58" ht="23" customHeight="1">
       <x:c r="A58" s="3" t="str">
@@ -2341,9 +2168,6 @@
       <x:c r="H58" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I58" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="59" ht="23" customHeight="1">
       <x:c r="A59" s="3" t="str">
@@ -2370,9 +2194,6 @@
       <x:c r="H59" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I59" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="60" ht="23" customHeight="1">
       <x:c r="A60" s="3" t="str">
@@ -2399,9 +2220,6 @@
       <x:c r="H60" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I60" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="61" ht="23" customHeight="1">
       <x:c r="A61" s="3" t="str">
@@ -2428,9 +2246,6 @@
       <x:c r="H61" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I61" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="62" ht="23" customHeight="1">
       <x:c r="A62" s="3" t="str">
@@ -2457,9 +2272,6 @@
       <x:c r="H62" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I62" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="63" ht="23" customHeight="1">
       <x:c r="A63" s="3" t="str">
@@ -2486,9 +2298,6 @@
       <x:c r="H63" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I63" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="64" ht="23" customHeight="1">
       <x:c r="A64" s="3" t="str">
@@ -2515,9 +2324,6 @@
       <x:c r="H64" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I64" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="65" ht="23" customHeight="1">
       <x:c r="A65" s="3" t="str">
@@ -2544,9 +2350,6 @@
       <x:c r="H65" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I65" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="66" ht="23" customHeight="1">
       <x:c r="A66" s="3" t="str">
@@ -2573,9 +2376,6 @@
       <x:c r="H66" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I66" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="67" ht="23" customHeight="1">
       <x:c r="A67" s="3" t="str">
@@ -2602,9 +2402,6 @@
       <x:c r="H67" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I67" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="68" ht="23" customHeight="1">
       <x:c r="A68" s="3" t="str">
@@ -2631,9 +2428,6 @@
       <x:c r="H68" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I68" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="69" ht="23" customHeight="1">
       <x:c r="A69" s="3" t="str">
@@ -2660,9 +2454,6 @@
       <x:c r="H69" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I69" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="70" ht="23" customHeight="1">
       <x:c r="A70" s="3" t="str">
@@ -2689,9 +2480,6 @@
       <x:c r="H70" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I70" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="71" ht="23" customHeight="1">
       <x:c r="A71" s="3" t="str">
@@ -2718,9 +2506,6 @@
       <x:c r="H71" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I71" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="72" ht="23" customHeight="1">
       <x:c r="A72" s="3" t="str">
@@ -2747,9 +2532,6 @@
       <x:c r="H72" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I72" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="73" ht="23" customHeight="1">
       <x:c r="A73" s="3" t="str">
@@ -2776,9 +2558,6 @@
       <x:c r="H73" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I73" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="74" ht="23" customHeight="1">
       <x:c r="A74" s="3" t="str">
@@ -2805,9 +2584,6 @@
       <x:c r="H74" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I74" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="75" ht="23" customHeight="1">
       <x:c r="A75" s="3" t="str">
@@ -2834,9 +2610,6 @@
       <x:c r="H75" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I75" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="76" ht="23" customHeight="1">
       <x:c r="A76" s="3" t="str">
@@ -2863,9 +2636,6 @@
       <x:c r="H76" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I76" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="77" ht="23" customHeight="1">
       <x:c r="A77" s="3" t="str">
@@ -2892,9 +2662,6 @@
       <x:c r="H77" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I77" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="78" ht="23" customHeight="1">
       <x:c r="A78" s="3" t="str">
@@ -2921,9 +2688,6 @@
       <x:c r="H78" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I78" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="79" ht="23" customHeight="1">
       <x:c r="A79" s="3" t="str">
@@ -2950,9 +2714,6 @@
       <x:c r="H79" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I79" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="80" ht="23" customHeight="1">
       <x:c r="A80" s="3" t="str">
@@ -2979,9 +2740,6 @@
       <x:c r="H80" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I80" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="81" ht="23" customHeight="1">
       <x:c r="A81" s="3" t="str">
@@ -3008,9 +2766,6 @@
       <x:c r="H81" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I81" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="82" ht="23" customHeight="1">
       <x:c r="A82" s="3" t="str">
@@ -3037,9 +2792,6 @@
       <x:c r="H82" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I82" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="83" ht="23" customHeight="1">
       <x:c r="A83" s="3" t="str">
@@ -3066,9 +2818,6 @@
       <x:c r="H83" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I83" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="84" ht="23" customHeight="1">
       <x:c r="A84" s="3" t="str">
@@ -3095,9 +2844,6 @@
       <x:c r="H84" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I84" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="85" ht="23" customHeight="1">
       <x:c r="A85" s="3" t="str">
@@ -3124,9 +2870,6 @@
       <x:c r="H85" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I85" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="86" ht="23" customHeight="1">
       <x:c r="A86" s="3" t="str">
@@ -3153,9 +2896,6 @@
       <x:c r="H86" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I86" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="87" ht="23" customHeight="1">
       <x:c r="A87" s="3" t="str">
@@ -3182,9 +2922,6 @@
       <x:c r="H87" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I87" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="88" ht="23" customHeight="1">
       <x:c r="A88" s="3" t="str">
@@ -3211,9 +2948,6 @@
       <x:c r="H88" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I88" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="89" ht="23" customHeight="1">
       <x:c r="A89" s="3" t="str">
@@ -3240,9 +2974,6 @@
       <x:c r="H89" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I89" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="90" ht="23" customHeight="1">
       <x:c r="A90" s="3" t="str">
@@ -3269,9 +3000,6 @@
       <x:c r="H90" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I90" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="91" ht="23" customHeight="1">
       <x:c r="A91" s="3" t="str">
@@ -3298,9 +3026,6 @@
       <x:c r="H91" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I91" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="92" ht="23" customHeight="1">
       <x:c r="A92" s="3" t="str">
@@ -3327,9 +3052,6 @@
       <x:c r="H92" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I92" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="93" ht="23" customHeight="1">
       <x:c r="A93" s="3" t="str">
@@ -3356,9 +3078,6 @@
       <x:c r="H93" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I93" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="94" ht="23" customHeight="1">
       <x:c r="A94" s="3" t="str">
@@ -3385,9 +3104,6 @@
       <x:c r="H94" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I94" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="95" ht="23" customHeight="1">
       <x:c r="A95" s="3" t="str">
@@ -3414,9 +3130,6 @@
       <x:c r="H95" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I95" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="96" ht="23" customHeight="1">
       <x:c r="A96" s="3" t="str">
@@ -3443,9 +3156,6 @@
       <x:c r="H96" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I96" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="97" ht="23" customHeight="1">
       <x:c r="A97" s="3" t="str">
@@ -3472,9 +3182,6 @@
       <x:c r="H97" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I97" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="98" ht="23" customHeight="1">
       <x:c r="A98" s="3" t="str">
@@ -3501,9 +3208,6 @@
       <x:c r="H98" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I98" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="99" ht="23" customHeight="1">
       <x:c r="A99" s="3" t="str">
@@ -3530,9 +3234,6 @@
       <x:c r="H99" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I99" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="100" ht="23" customHeight="1">
       <x:c r="A100" s="3" t="str">
@@ -3559,9 +3260,6 @@
       <x:c r="H100" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I100" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
     <x:row r="101" ht="23" customHeight="1">
       <x:c r="A101" s="3" t="str">
@@ -3588,14 +3286,11 @@
       <x:c r="H101" s="6" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I101" s="3" t="str">
-        <x:v>modeled</x:v>
-      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67af73a5c4fc41a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddf1ba8b38504691"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4155,7 +3850,7 @@
     <x:row r="27" ht="25" customHeight="1">
       <x:c r="A27" s="14"/>
       <x:c r="B27" s="25" t="str">
-        <x:v>Детальные записи смоделированы. Итоговые показатели — из презентации проекта.</x:v>
+        <x:v>Выборка: 100 ответов. Критерий: названы не менее трёх народов.</x:v>
       </x:c>
       <x:c r="C27" s="14"/>
       <x:c r="D27" s="14"/>
@@ -4174,7 +3869,7 @@
     <x:row r="28" ht="25" customHeight="1">
       <x:c r="A28" s="14"/>
       <x:c r="B28" s="25" t="str">
-        <x:v>Выборка: 100 ответов. Критерий: названы не менее трёх народов.</x:v>
+        <x:v>Источник итогового показателя: «Мозаика Культур 2 (1)», слайд 14.</x:v>
       </x:c>
       <x:c r="C28" s="14"/>
       <x:c r="D28" s="14"/>
@@ -4192,9 +3887,7 @@
     </x:row>
     <x:row r="29" ht="25" customHeight="1">
       <x:c r="A29" s="14"/>
-      <x:c r="B29" s="25" t="str">
-        <x:v>Контрольная доля: презентация «Мозаика Культур 2 (1)», слайд 14.</x:v>
-      </x:c>
+      <x:c r="B29" s="14"/>
       <x:c r="C29" s="14"/>
       <x:c r="D29" s="14"/>
       <x:c r="E29" s="14"/>
@@ -4466,6 +4159,6 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41173d6e4541441e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d8320716ec04ef5"/>
 </x:worksheet>
 </file>
</xml_diff>